<commit_message>
Make final table with bootstrap uncertainty propoortions.
</commit_message>
<xml_diff>
--- a/outputs/final-scores-compiled/overall-vulnerability-rankings/overall_vulnerability_scores_uscar.xlsx
+++ b/outputs/final-scores-compiled/overall-vulnerability-rankings/overall_vulnerability_scores_uscar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\Caribbean-CVA\outputs\final-scores-compiled\overall-vulnerability-rankings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{59D9BF06-ED2A-4B4B-A940-3D9FA47831EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1765CE5-75D9-4E96-88BE-43B3A01FA1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37515" yWindow="2280" windowWidth="17970" windowHeight="12780" xr2:uid="{DCDD4FB4-8ADE-44C2-82D3-D9D1986B6C86}"/>
+    <workbookView xWindow="15810" yWindow="1830" windowWidth="11490" windowHeight="13350" xr2:uid="{DCDD4FB4-8ADE-44C2-82D3-D9D1986B6C86}"/>
   </bookViews>
   <sheets>
     <sheet name="overall_vulnerability_scores_us" sheetId="1" r:id="rId1"/>
@@ -127,10 +127,10 @@
     <t>Vuln rank</t>
   </si>
   <si>
-    <t>Diadima</t>
-  </si>
-  <si>
     <t>Atlantic herring</t>
+  </si>
+  <si>
+    <t>Diadema</t>
   </si>
 </sst>
 </file>
@@ -790,182 +790,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="32">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <fill>
         <patternFill>
@@ -1011,7 +836,42 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1386,10 +1246,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2">
         <v>4</v>
@@ -1415,7 +1275,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="2">
         <v>4</v>
@@ -1441,7 +1301,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="14">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="14">
         <v>4</v>
@@ -1467,7 +1327,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" s="2">
         <v>3</v>
@@ -1493,7 +1353,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C6" s="2">
         <v>3</v>
@@ -1519,7 +1379,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C7" s="2">
         <v>4</v>
@@ -1545,7 +1405,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="2">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2">
         <v>4</v>
@@ -1571,7 +1431,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C9" s="2">
         <v>4</v>
@@ -1597,7 +1457,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="2">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C10" s="2">
         <v>4</v>
@@ -1623,7 +1483,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C11" s="2">
         <v>4</v>
@@ -1649,7 +1509,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="14">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C12" s="14">
         <v>4</v>
@@ -1675,7 +1535,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C13" s="2">
         <v>3</v>
@@ -1701,7 +1561,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C14" s="2">
         <v>3</v>
@@ -1727,7 +1587,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C15" s="2">
         <v>3</v>
@@ -1753,7 +1613,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C16" s="2">
         <v>4</v>
@@ -1779,7 +1639,7 @@
         <v>18</v>
       </c>
       <c r="B17" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C17" s="2">
         <v>4</v>
@@ -1805,7 +1665,7 @@
         <v>19</v>
       </c>
       <c r="B18" s="14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C18" s="14">
         <v>4</v>
@@ -1828,10 +1688,10 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B19" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19" s="2">
         <v>3</v>
@@ -1857,7 +1717,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C20" s="2">
         <v>3</v>
@@ -1883,7 +1743,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C21" s="2">
         <v>2</v>
@@ -1935,7 +1795,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C23" s="2">
         <v>1</v>
@@ -1961,7 +1821,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C24" s="2">
         <v>1</v>
@@ -2013,7 +1873,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C26" s="4">
         <v>1</v>
@@ -2038,56 +1898,50 @@
       <c r="A27" s="5"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H1:H1048576 F1:F1048576 D1:D1048576">
-    <cfRule type="containsText" dxfId="11" priority="12" operator="containsText" text="Very High">
+  <conditionalFormatting sqref="C1:C1048576 E1:E1048576">
+    <cfRule type="cellIs" dxfId="11" priority="5" operator="equal">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="6" operator="equal">
+      <formula>2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="7" operator="equal">
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
+      <formula>4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:D1048576 F1:F1048576 H1:H1048576">
+    <cfRule type="cellIs" dxfId="7" priority="9" operator="equal">
+      <formula>"Low"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="10" operator="equal">
+      <formula>"Moderate"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="11" operator="equal">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="12" operator="containsText" text="Very High">
       <formula>NOT(ISERROR(SEARCH("Very High",D1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H1048576 F1:F1048576 D1:D1048576">
-    <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
-      <formula>"High"</formula>
+  <conditionalFormatting sqref="G2:G26">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="between">
+      <formula>6.5</formula>
+      <formula>9.5</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H1048576 F1:F1048576 D1:D1048576">
-    <cfRule type="cellIs" dxfId="9" priority="10" operator="equal">
-      <formula>"Moderate"</formula>
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="between">
+      <formula>3.5</formula>
+      <formula>6.5</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H1048576 F1:F1048576 D1:D1048576">
-    <cfRule type="cellIs" dxfId="8" priority="9" operator="equal">
-      <formula>"Low"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C1048576 E1:E1048576">
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
-      <formula>4</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThanOrEqual">
       <formula>3</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
-      <formula>2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
-      <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G1048576">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="greaterThanOrEqual">
       <formula>12</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G26">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThanOrEqual">
-      <formula>3</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="between">
-      <formula>3.5</formula>
-      <formula>6.5</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="between">
-      <formula>6.5</formula>
-      <formula>9.5</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>